<commit_message>
Preparação de entrega final
</commit_message>
<xml_diff>
--- a/docs/Cronograma_ProjetoAplicadoIII.xlsx
+++ b/docs/Cronograma_ProjetoAplicadoIII.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Ricardo\Documents\ESTUDO\Mackenzie\04_Sem\PROJ_III\Projeto-Aplicado3-Grupo12\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93B0970F-7C2E-4DB9-A4AE-896A71F5884C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED168E0D-2184-450F-9A2D-B6DD1EE4ADD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23080" yWindow="2950" windowWidth="27280" windowHeight="21700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2110" yWindow="4910" windowWidth="27280" windowHeight="21700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Controlador de projetos" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="49">
   <si>
     <t>Categoria</t>
   </si>
@@ -128,9 +128,6 @@
   </si>
   <si>
     <t>Vídeo</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Projeto Aplicado 3 - Grupo 12 - 2026.1</t>
@@ -1482,7 +1479,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="65.150000000000006" customHeight="1">
       <c r="B1" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C1" s="6"/>
       <c r="D1" s="6"/>
@@ -1491,7 +1488,7 @@
       <c r="A2" s="2"/>
       <c r="B2" s="6"/>
       <c r="C2" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="3"/>
@@ -1534,7 +1531,7 @@
     </row>
     <row r="5" spans="1:12" ht="30" customHeight="1">
       <c r="B5" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>25</v>
@@ -1569,7 +1566,7 @@
     </row>
     <row r="6" spans="1:12" ht="30" customHeight="1">
       <c r="B6" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C6" s="12" t="s">
         <v>23</v>
@@ -1604,7 +1601,7 @@
     </row>
     <row r="7" spans="1:12" ht="30" customHeight="1">
       <c r="B7" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>24</v>
@@ -1639,7 +1636,7 @@
     </row>
     <row r="8" spans="1:12" ht="30" customHeight="1" thickBot="1">
       <c r="B8" s="22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="22" t="s">
         <v>22</v>
@@ -1674,7 +1671,7 @@
     </row>
     <row r="9" spans="1:12" ht="30" customHeight="1">
       <c r="B9" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C9" s="12" t="s">
         <v>25</v>
@@ -1709,7 +1706,7 @@
     </row>
     <row r="10" spans="1:12" ht="30" customHeight="1">
       <c r="B10" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>23</v>
@@ -1744,7 +1741,7 @@
     </row>
     <row r="11" spans="1:12" ht="30" customHeight="1">
       <c r="B11" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>25</v>
@@ -1779,7 +1776,7 @@
     </row>
     <row r="12" spans="1:12" ht="30" customHeight="1">
       <c r="B12" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C12" s="12" t="s">
         <v>24</v>
@@ -1814,7 +1811,7 @@
     </row>
     <row r="13" spans="1:12" ht="30" customHeight="1">
       <c r="B13" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C13" s="12" t="s">
         <v>22</v>
@@ -1849,7 +1846,7 @@
     </row>
     <row r="14" spans="1:12" ht="30" customHeight="1" thickBot="1">
       <c r="B14" s="22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C14" s="22" t="s">
         <v>24</v>
@@ -1884,7 +1881,7 @@
     </row>
     <row r="15" spans="1:12" ht="30" customHeight="1">
       <c r="B15" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="12" t="s">
         <v>25</v>
@@ -1919,7 +1916,7 @@
     </row>
     <row r="16" spans="1:12" ht="30" customHeight="1">
       <c r="B16" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" s="12" t="s">
         <v>24</v>
@@ -1954,7 +1951,7 @@
     </row>
     <row r="17" spans="2:12" ht="30" customHeight="1">
       <c r="B17" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C17" s="12" t="s">
         <v>23</v>
@@ -1989,7 +1986,7 @@
     </row>
     <row r="18" spans="2:12" ht="30" customHeight="1">
       <c r="B18" s="12" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C18" s="12" t="s">
         <v>23</v>
@@ -2024,7 +2021,7 @@
     </row>
     <row r="19" spans="2:12" ht="30" customHeight="1" thickBot="1">
       <c r="B19" s="22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C19" s="22" t="s">
         <v>22</v>
@@ -2059,10 +2056,10 @@
     </row>
     <row r="20" spans="2:12" ht="30" customHeight="1">
       <c r="B20" s="12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>19</v>
@@ -2080,19 +2077,24 @@
         <f>IF(COUNTA('Controlador de projetos'!$F20,'Controlador de projetos'!$G20)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F20,'Controlador de projetos'!$G20,FALSE)+1)</f>
         <v>22</v>
       </c>
-      <c r="I20" s="14"/>
-      <c r="J20" s="13"/>
-      <c r="K20" s="15" t="s">
-        <v>27</v>
+      <c r="I20" s="14">
+        <v>46144</v>
+      </c>
+      <c r="J20" s="13">
+        <v>46146</v>
+      </c>
+      <c r="K20" s="15">
+        <f>IF(COUNTA('Controlador de projetos'!$I20,'Controlador de projetos'!$J20)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I20,'Controlador de projetos'!$J20,FALSE)+1)</f>
+        <v>3</v>
       </c>
       <c r="L20" s="12"/>
     </row>
     <row r="21" spans="2:12" ht="30" customHeight="1">
       <c r="B21" s="12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C21" s="12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>19</v>
@@ -2110,20 +2112,24 @@
         <f>IF(COUNTA('Controlador de projetos'!$F21,'Controlador de projetos'!$G21)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F21,'Controlador de projetos'!$G21,FALSE))</f>
         <v>21</v>
       </c>
-      <c r="I21" s="14"/>
-      <c r="J21" s="13"/>
-      <c r="K21" s="15" t="str">
-        <f>IF(COUNTA('Controlador de projetos'!$I21,'Controlador de projetos'!$J21)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I21,'Controlador de projetos'!$J21,FALSE))</f>
-        <v/>
+      <c r="I21" s="14">
+        <v>46144</v>
+      </c>
+      <c r="J21" s="13">
+        <v>46147</v>
+      </c>
+      <c r="K21" s="15">
+        <f>IF(COUNTA('Controlador de projetos'!$I21,'Controlador de projetos'!$J21)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I21,'Controlador de projetos'!$J21,FALSE)+1)</f>
+        <v>4</v>
       </c>
       <c r="L21" s="12"/>
     </row>
     <row r="22" spans="2:12" ht="30" customHeight="1">
       <c r="B22" s="12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>19</v>
@@ -2141,20 +2147,24 @@
         <f>IF(COUNTA('Controlador de projetos'!$F22,'Controlador de projetos'!$G22)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F22,'Controlador de projetos'!$G22,FALSE))</f>
         <v>21</v>
       </c>
-      <c r="I22" s="14"/>
-      <c r="J22" s="13"/>
-      <c r="K22" s="15" t="str">
-        <f>IF(COUNTA('Controlador de projetos'!$I22,'Controlador de projetos'!$J22)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I22,'Controlador de projetos'!$J22,FALSE))</f>
-        <v/>
+      <c r="I22" s="14">
+        <v>46144</v>
+      </c>
+      <c r="J22" s="13">
+        <v>46147</v>
+      </c>
+      <c r="K22" s="15">
+        <f>IF(COUNTA('Controlador de projetos'!$I22,'Controlador de projetos'!$J22)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I22,'Controlador de projetos'!$J22,FALSE)+1)</f>
+        <v>4</v>
       </c>
       <c r="L22" s="12"/>
     </row>
     <row r="23" spans="2:12" ht="30" customHeight="1">
       <c r="B23" s="12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>19</v>
@@ -2172,20 +2182,24 @@
         <f>IF(COUNTA('Controlador de projetos'!$F23,'Controlador de projetos'!$G23)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F23,'Controlador de projetos'!$G23,FALSE))</f>
         <v>21</v>
       </c>
-      <c r="I23" s="14"/>
-      <c r="J23" s="13"/>
-      <c r="K23" s="15" t="str">
-        <f>IF(COUNTA('Controlador de projetos'!$I23,'Controlador de projetos'!$J23)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I23,'Controlador de projetos'!$J23,FALSE))</f>
-        <v/>
+      <c r="I23" s="14">
+        <v>46148</v>
+      </c>
+      <c r="J23" s="13">
+        <v>46150</v>
+      </c>
+      <c r="K23" s="15">
+        <f>IF(COUNTA('Controlador de projetos'!$I23,'Controlador de projetos'!$J23)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I23,'Controlador de projetos'!$J23,FALSE)+1)</f>
+        <v>3</v>
       </c>
       <c r="L23" s="12"/>
     </row>
     <row r="24" spans="2:12" ht="30" customHeight="1">
       <c r="B24" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>19</v>
@@ -2203,11 +2217,15 @@
         <f>IF(COUNTA('Controlador de projetos'!$F24,'Controlador de projetos'!$G24)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F24,'Controlador de projetos'!$G24,FALSE)+1)</f>
         <v>22</v>
       </c>
-      <c r="I24" s="14"/>
-      <c r="J24" s="13"/>
-      <c r="K24" s="15" t="str">
+      <c r="I24" s="14">
+        <v>46151</v>
+      </c>
+      <c r="J24" s="13">
+        <v>46154</v>
+      </c>
+      <c r="K24" s="15">
         <f>IF(COUNTA('Controlador de projetos'!$I24,'Controlador de projetos'!$J24)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I24,'Controlador de projetos'!$J24,FALSE)+1)</f>
-        <v/>
+        <v>4</v>
       </c>
       <c r="L24" s="12"/>
     </row>
@@ -2216,7 +2234,7 @@
         <v>26</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>19</v>
@@ -2234,20 +2252,24 @@
         <f>IF(COUNTA('Controlador de projetos'!$F25,'Controlador de projetos'!$G25)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F25,'Controlador de projetos'!$G25,FALSE)+1)</f>
         <v>22</v>
       </c>
-      <c r="I25" s="14"/>
-      <c r="J25" s="13"/>
-      <c r="K25" s="15" t="str">
+      <c r="I25" s="14">
+        <v>46155</v>
+      </c>
+      <c r="J25" s="13">
+        <v>46161</v>
+      </c>
+      <c r="K25" s="15">
         <f>IF(COUNTA('Controlador de projetos'!$I25,'Controlador de projetos'!$J25)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I25,'Controlador de projetos'!$J25,FALSE)+1)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="L25" s="12"/>
     </row>
     <row r="26" spans="2:12" ht="30" customHeight="1" thickBot="1">
       <c r="B26" s="22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D26" s="22" t="s">
         <v>19</v>
@@ -2265,11 +2287,15 @@
         <f>IF(COUNTA('Controlador de projetos'!$F26,'Controlador de projetos'!$G26)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$F26,'Controlador de projetos'!$G26,FALSE)+1)</f>
         <v>22</v>
       </c>
-      <c r="I26" s="27"/>
-      <c r="J26" s="23"/>
-      <c r="K26" s="26" t="str">
+      <c r="I26" s="27">
+        <v>46155</v>
+      </c>
+      <c r="J26" s="23">
+        <v>46161</v>
+      </c>
+      <c r="K26" s="26">
         <f>IF(COUNTA('Controlador de projetos'!$I26,'Controlador de projetos'!$J26)&lt;&gt;2,"",DAYS360('Controlador de projetos'!$I26,'Controlador de projetos'!$J26,FALSE)+1)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="L26" s="22"/>
     </row>

</xml_diff>